<commit_message>
Update comparative execution records with Task Outcome and Manifest Ground-Truth grading
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -10,7 +10,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="195">
   <si>
     <t xml:space="preserve">Timestamp (UTC)</t>
   </si>
@@ -264,6 +264,69 @@
     <t xml:space="preserve">Rejected (SOLVER_INFEASIBLE)</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-10-08 09:57:48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bhai mujhe AWS pe aath core aur solah gig RAM wala setup chahiye, budget teen sau dollar tak rakhna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feasible against checked constraints (Unverified LLM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08 10:01:56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bhai AWS aur GCP dono pe disaster recovery chahiye, 99.99 percent uptime, latency pachaas millisecond se kam, budget chhe sau dollar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08 10:02:43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dynamic scaling for 300 Mbps peak workload with target CPU 70 percent and strict maximum CPU ceiling of 60 percent under 1500 dollar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conflicting requirements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08 10:03:40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I need a server on AWS with 8 vCPUs and 16GB RAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08 10:04:18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deploy a massive database requiring 64 vCPUs and 256GB RAM on AWS for under 10 dollar a month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08 10:04:44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Train a transformer model on 8 H100 GPUs for two weeks and tell me the cheapest option</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOT_EVALUABLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unsupported workload domain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08 10:22:02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bhai AWS pe 8 vCPU aur 16GB RAM ka setup lagade 300 dollar per month ke andar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08 10:22:28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I want to run a web backend with 8 vCPUs and 16GB RAM on AWS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invalid output structure (No VMs)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Query ID</t>
   </si>
   <si>
@@ -432,10 +495,37 @@
     <t xml:space="preserve">Q16</t>
   </si>
   <si>
+    <t xml:space="preserve">Q17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOT_EVALUABLE | —</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q24</t>
+  </si>
+  <si>
     <t xml:space="preserve">NEURASYM 4-WAY PARADIGM BENCHMARK EXECUTIVE SUMMARY</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated at: 2026-10-08 09:56:00 UTC</t>
+    <t xml:space="preserve">Generated at: 2026-10-08 10:22:28 UTC</t>
   </si>
   <si>
     <t xml:space="preserve">Paradigm Evaluation Mode</t>
@@ -462,7 +552,7 @@
     <t xml:space="preserve">Groq API (openai/gpt-oss-120b)</t>
   </si>
   <si>
-    <t xml:space="preserve">912.51 ms</t>
+    <t xml:space="preserve">608.34 ms</t>
   </si>
   <si>
     <t xml:space="preserve">Mode 2: Schema-Constrained LLM</t>
@@ -471,7 +561,7 @@
     <t xml:space="preserve">Groq API (Strict Pydantic JSON)</t>
   </si>
   <si>
-    <t xml:space="preserve">296.44 ms</t>
+    <t xml:space="preserve">197.63 ms</t>
   </si>
   <si>
     <t xml:space="preserve">Mode 3: Pure Symbolic Pipeline</t>
@@ -480,7 +570,7 @@
     <t xml:space="preserve">Local Solvers (HiGHS / PSO / Z3)</t>
   </si>
   <si>
-    <t xml:space="preserve">5.47 ms</t>
+    <t xml:space="preserve">3.65 ms</t>
   </si>
   <si>
     <t xml:space="preserve">Mode 4: Full Neuro-Symbolic</t>
@@ -489,7 +579,7 @@
     <t xml:space="preserve">Local Solvers + NVIDIA Explainer</t>
   </si>
   <si>
-    <t xml:space="preserve">2.17 ms</t>
+    <t xml:space="preserve">1.45 ms</t>
   </si>
   <si>
     <t xml:space="preserve">CORE ARCHITECTURAL TAKEAWAYS</t>
@@ -2936,6 +3026,1126 @@
         <v>55</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="B66" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="C66" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D66" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="E66" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F66" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G66" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I66" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="J66" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K66" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="B67" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="C67" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D67" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E67" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F67" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G67" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I67" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="J67" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K67" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="B68" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D68" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="E68" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F68" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G68" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H68" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I68" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="J68" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K68" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="B69" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="C69" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D69" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="E69" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F69" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G69" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I69" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="J69" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K69" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D70" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F70" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G70" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H70" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I70" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="J70" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K70" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C71" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D71" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F71" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G71" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H71" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I71" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="J71" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K71" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D72" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F72" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G72" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H72" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I72" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J72" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K72" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C73" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F73" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G73" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H73" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I73" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J73" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K73" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="B74" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D74" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="E74" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F74" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G74" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H74" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I74" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="J74" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K74" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="B75" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="C75" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D75" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E75" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F75" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G75" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H75" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I75" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="J75" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K75" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="B76" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D76" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="E76" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F76" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G76" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H76" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I76" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="J76" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K76" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="B77" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="C77" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D77" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="E77" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F77" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G77" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H77" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I77" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="J77" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K77" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F78" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G78" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H78" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I78" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="J78" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K78" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C79" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F79" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G79" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H79" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I79" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="J79" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K79" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E80" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F80" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G80" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H80" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I80" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J80" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K80" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C81" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E81" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F81" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G81" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H81" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="I81" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="J81" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K81" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="B82" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D82" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="E82" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F82" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G82" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H82" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I82" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="J82" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K82" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="B83" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="C83" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D83" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E83" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F83" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G83" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H83" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I83" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="J83" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K83" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="B84" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D84" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="E84" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F84" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G84" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H84" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I84" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="J84" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K84" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="B85" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="C85" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D85" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="E85" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F85" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G85" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H85" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I85" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="J85" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K85" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D86" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E86" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F86" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G86" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H86" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I86" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="J86" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K86" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C87" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D87" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E87" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F87" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G87" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H87" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I87" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="J87" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K87" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D88" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E88" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F88" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G88" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H88" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I88" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J88" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K88" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C89" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D89" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E89" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F89" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G89" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H89" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I89" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="J89" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K89" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="B90" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D90" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="E90" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F90" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G90" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H90" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I90" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="J90" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K90" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="B91" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="C91" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D91" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E91" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F91" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G91" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H91" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I91" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="J91" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K91" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="B92" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D92" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="E92" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F92" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G92" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H92" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I92" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="J92" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K92" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="B93" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="C93" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D93" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="E93" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F93" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G93" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H93" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I93" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="J93" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K93" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D94" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E94" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F94" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G94" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H94" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I94" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="J94" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K94" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C95" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D95" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E95" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F95" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G95" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H95" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I95" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="J95" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K95" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B96" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C96" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D96" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E96" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F96" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G96" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H96" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I96" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J96" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K96" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C97" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E97" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F97" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G97" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H97" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="I97" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="J97" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K97" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -2958,597 +4168,877 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>88</v>
+        <v>109</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>92</v>
+        <v>113</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>94</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>97</v>
+        <v>118</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>98</v>
+        <v>119</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>101</v>
+        <v>122</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>101</v>
+        <v>122</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>103</v>
+        <v>124</v>
       </c>
       <c r="B3" s="0" t="s">
         <v>41</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>104</v>
+        <v>125</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>105</v>
+        <v>126</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>98</v>
+        <v>119</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>106</v>
+        <v>127</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="K3" s="0" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>50</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>98</v>
+        <v>119</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>115</v>
+        <v>136</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>116</v>
+        <v>137</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
-        <v>117</v>
+        <v>138</v>
       </c>
       <c r="B5" s="0" t="s">
         <v>50</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>98</v>
-      </c>
       <c r="F5" s="5" t="s">
-        <v>120</v>
+        <v>141</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>121</v>
+        <v>142</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>122</v>
+        <v>143</v>
       </c>
       <c r="K5" s="0" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>123</v>
+        <v>144</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>41</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="B7" s="0" t="s">
         <v>60</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="K7" s="0" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>63</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="B9" s="0" t="s">
         <v>66</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>12</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>132</v>
+        <v>153</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>41</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="K11" s="0" t="s">
-        <v>102</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>133</v>
+        <v>154</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>50</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="B13" s="0" t="s">
         <v>50</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="K13" s="0" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
-        <v>135</v>
+        <v>156</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>50</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="B15" s="0" t="s">
         <v>50</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="K15" s="0" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="s">
-        <v>138</v>
+        <v>159</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>80</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="s">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="B17" s="0" t="s">
         <v>80</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>125</v>
+        <v>146</v>
       </c>
       <c r="K17" s="0" t="s">
-        <v>110</v>
+        <v>131</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="K18" s="6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="K19" s="0" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="s">
+        <v>163</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="K20" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="K21" s="0" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="J23" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="K23" s="0" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="I25" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="K25" s="0" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -3568,7 +5058,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3578,7 +5068,7 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>141</v>
+        <v>171</v>
       </c>
       <c r="B2" s="0"/>
       <c r="C2" s="0"/>
@@ -3596,102 +5086,102 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>142</v>
+        <v>172</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>143</v>
+        <v>173</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>144</v>
+        <v>174</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>145</v>
+        <v>175</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>146</v>
+        <v>176</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>147</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
-        <v>148</v>
+        <v>178</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>149</v>
+        <v>179</v>
       </c>
       <c r="C5" s="5">
-        <v>16</v>
-      </c>
-      <c r="D5" s="0">
-        <v>0</v>
+        <v>24</v>
+      </c>
+      <c r="D5" s="3">
+        <v>2</v>
       </c>
       <c r="E5" s="4">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>150</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>151</v>
+        <v>181</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>152</v>
+        <v>182</v>
       </c>
       <c r="C6" s="5">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D6" s="3">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E6" s="4">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>153</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>154</v>
+        <v>184</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>155</v>
+        <v>185</v>
       </c>
       <c r="C7" s="5">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D7" s="3">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="E7" s="4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>156</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>157</v>
+        <v>187</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>158</v>
+        <v>188</v>
       </c>
       <c r="C8" s="5">
+        <v>24</v>
+      </c>
+      <c r="D8" s="3">
+        <v>8</v>
+      </c>
+      <c r="E8" s="4">
         <v>16</v>
       </c>
-      <c r="D8" s="3">
-        <v>5</v>
-      </c>
-      <c r="E8" s="4">
-        <v>11</v>
-      </c>
       <c r="F8" s="5" t="s">
-        <v>159</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9">
@@ -3704,7 +5194,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>160</v>
+        <v>190</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -3714,7 +5204,7 @@
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>161</v>
+        <v>191</v>
       </c>
       <c r="B11" s="0"/>
       <c r="C11" s="0"/>
@@ -3724,7 +5214,7 @@
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>162</v>
+        <v>192</v>
       </c>
       <c r="B12" s="0"/>
       <c r="C12" s="0"/>
@@ -3734,7 +5224,7 @@
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>163</v>
+        <v>193</v>
       </c>
       <c r="B13" s="0"/>
       <c r="C13" s="0"/>
@@ -3744,7 +5234,7 @@
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
-        <v>164</v>
+        <v>194</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>

</xml_diff>

<commit_message>
Update test benchmark results for 300 Mbps scaling and H100 GPU queries
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -10,7 +10,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="206">
   <si>
     <t xml:space="preserve">Timestamp (UTC)</t>
   </si>
@@ -327,6 +327,30 @@
     <t xml:space="preserve">Invalid output structure (No VMs)</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-10-08 10:23:19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rejected (NEEDS_REVIEW)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STAGE 1 (PARSER_FAILED): RESULT: PARSER_FAILED -- no archetype could be constructed from this input.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08 10:36:38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dynamic scaling for 300 Mbps peak workload with target CPU 70% under</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALID_PLAN (Feasible against checked constraints)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-08 10:36:58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNPARSEABLE (NEEDS_REVIEW)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Query ID</t>
   </si>
   <si>
@@ -522,10 +546,19 @@
     <t xml:space="preserve">Q24</t>
   </si>
   <si>
+    <t xml:space="preserve">Q25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q27</t>
+  </si>
+  <si>
     <t xml:space="preserve">NEURASYM 4-WAY PARADIGM BENCHMARK EXECUTIVE SUMMARY</t>
   </si>
   <si>
-    <t xml:space="preserve">Generated at: 2026-10-08 10:22:28 UTC</t>
+    <t xml:space="preserve">Generated at: 2026-10-08 10:36:58 UTC</t>
   </si>
   <si>
     <t xml:space="preserve">Paradigm Evaluation Mode</t>
@@ -552,7 +585,7 @@
     <t xml:space="preserve">Groq API (openai/gpt-oss-120b)</t>
   </si>
   <si>
-    <t xml:space="preserve">608.34 ms</t>
+    <t xml:space="preserve">540.74 ms</t>
   </si>
   <si>
     <t xml:space="preserve">Mode 2: Schema-Constrained LLM</t>
@@ -561,7 +594,7 @@
     <t xml:space="preserve">Groq API (Strict Pydantic JSON)</t>
   </si>
   <si>
-    <t xml:space="preserve">197.63 ms</t>
+    <t xml:space="preserve">175.67 ms</t>
   </si>
   <si>
     <t xml:space="preserve">Mode 3: Pure Symbolic Pipeline</t>
@@ -570,7 +603,7 @@
     <t xml:space="preserve">Local Solvers (HiGHS / PSO / Z3)</t>
   </si>
   <si>
-    <t xml:space="preserve">3.65 ms</t>
+    <t xml:space="preserve">3.24 ms</t>
   </si>
   <si>
     <t xml:space="preserve">Mode 4: Full Neuro-Symbolic</t>
@@ -579,7 +612,7 @@
     <t xml:space="preserve">Local Solvers + NVIDIA Explainer</t>
   </si>
   <si>
-    <t xml:space="preserve">1.45 ms</t>
+    <t xml:space="preserve">1.29 ms</t>
   </si>
   <si>
     <t xml:space="preserve">CORE ARCHITECTURAL TAKEAWAYS</t>
@@ -4146,6 +4179,426 @@
         <v>55</v>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="B98" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D98" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="E98" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F98" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G98" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H98" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I98" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="J98" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K98" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="B99" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="C99" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D99" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E99" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F99" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G99" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H99" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I99" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="J99" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K99" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="B100" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D100" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="E100" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F100" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G100" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H100" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I100" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="J100" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K100" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="B101" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="C101" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D101" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="E101" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F101" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G101" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H101" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I101" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="J101" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K101" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B102" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D102" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E102" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F102" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G102" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H102" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I102" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="J102" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K102" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B103" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C103" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D103" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E103" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F103" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G103" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H103" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I103" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J103" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K103" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B104" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C104" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D104" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E104" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F104" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G104" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H104" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I104" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="J104" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K104" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B105" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C105" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D105" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E105" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F105" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="G105" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H105" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="I105" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="J105" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="K105" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="B106" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D106" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="E106" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F106" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G106" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H106" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I106" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="J106" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K106" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="B107" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="C107" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D107" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E107" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F107" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G107" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H107" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I107" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="J107" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K107" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="B108" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="C108" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D108" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="E108" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F108" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G108" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H108" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I108" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="J108" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K108" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="B109" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="C109" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D109" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="E109" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="F109" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="G109" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H109" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I109" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="J109" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="K109" s="0" t="s">
+        <v>55</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -4168,877 +4621,982 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B3" s="0" t="s">
         <v>41</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="K3" s="0" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>50</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="H4" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="I4" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="I4" s="4" t="s">
-        <v>128</v>
-      </c>
       <c r="J4" s="7" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="K4" s="6" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="B5" s="0" t="s">
         <v>50</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="K5" s="0" t="s">
         <v>139</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="K5" s="0" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>41</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="B7" s="0" t="s">
         <v>60</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K7" s="0" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>63</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="B9" s="0" t="s">
         <v>66</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K9" s="0" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>12</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>41</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K11" s="0" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>50</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="B13" s="0" t="s">
         <v>50</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K13" s="0" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>50</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="B15" s="0" t="s">
         <v>50</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I15" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="K15" s="0" t="s">
         <v>158</v>
-      </c>
-      <c r="J15" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="K15" s="0" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>80</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B17" s="0" t="s">
         <v>80</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K17" s="0" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>85</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="B19" s="0" t="s">
         <v>88</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K19" s="0" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>90</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="B21" s="0" t="s">
         <v>93</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I21" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="K21" s="0" t="s">
         <v>158</v>
-      </c>
-      <c r="J21" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="K21" s="0" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>95</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="B23" s="0" t="s">
         <v>97</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K23" s="0" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>101</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="B25" s="0" t="s">
         <v>103</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="I25" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="J25" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="K25" s="0" t="s">
         <v>158</v>
       </c>
-      <c r="J25" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="K25" s="0" t="s">
-        <v>150</v>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="I26" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="K26" s="6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="J27" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="K27" s="0" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="s">
+        <v>180</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J28" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="K28" s="6" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -5058,7 +5616,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5068,7 +5626,7 @@
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="B2" s="0"/>
       <c r="C2" s="0"/>
@@ -5086,102 +5644,102 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="C5" s="5">
+        <v>27</v>
+      </c>
+      <c r="D5" s="3">
+        <v>3</v>
+      </c>
+      <c r="E5" s="4">
         <v>24</v>
       </c>
-      <c r="D5" s="3">
-        <v>2</v>
-      </c>
-      <c r="E5" s="4">
-        <v>22</v>
-      </c>
       <c r="F5" s="5" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="C6" s="5">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D6" s="3">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" s="4">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="C7" s="5">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D7" s="3">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E7" s="4">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="C8" s="5">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D8" s="3">
         <v>8</v>
       </c>
       <c r="E8" s="4">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9">
@@ -5194,7 +5752,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -5204,7 +5762,7 @@
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="B11" s="0"/>
       <c r="C11" s="0"/>
@@ -5214,7 +5772,7 @@
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="B12" s="0"/>
       <c r="C12" s="0"/>
@@ -5224,7 +5782,7 @@
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="B13" s="0"/>
       <c r="C13" s="0"/>
@@ -5234,7 +5792,7 @@
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>

</xml_diff>